<commit_message>
region grid: North West
</commit_message>
<xml_diff>
--- a/region/North-West-overview-grid.xlsx
+++ b/region/North-West-overview-grid.xlsx
@@ -150,7 +150,7 @@
     <row r="1" ht="20" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">H-E-B  |  Region Overview information — North West — generated 8/14/2026</t>
+          <t xml:space="preserve">H-E-B  |  Region Overview information — North West — generated 8/17/2026</t>
         </is>
       </c>
     </row>
@@ -1778,7 +1778,7 @@
       <c r="N17" s="5"/>
       <c r="O17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">12'3"' x 24'6"'</t>
+          <t xml:space="preserve">12'3" x 24'6"</t>
         </is>
       </c>
       <c r="P17" s="5"/>
@@ -2288,7 +2288,7 @@
       <c r="N22" s="4"/>
       <c r="O22" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">14'' x 48"'</t>
+          <t xml:space="preserve">14' x 48'</t>
         </is>
       </c>
       <c r="P22" s="4"/>
@@ -2594,7 +2594,7 @@
       <c r="N25" s="5"/>
       <c r="O25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">14'' x 48''</t>
+          <t xml:space="preserve">14' x 48'</t>
         </is>
       </c>
       <c r="P25" s="5"/>
@@ -2794,7 +2794,7 @@
       <c r="N27" s="5"/>
       <c r="O27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">14'' x 48''</t>
+          <t xml:space="preserve">14' x 48'</t>
         </is>
       </c>
       <c r="P27" s="5"/>
@@ -6294,7 +6294,7 @@
       <c r="N60" s="4"/>
       <c r="O60" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">16'' x 32"'</t>
+          <t xml:space="preserve">16' x 32'</t>
         </is>
       </c>
       <c r="P60" s="4"/>

</xml_diff>